<commit_message>
上新 Klimter - PlanetInspiredTraits（行星之子）
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2453,6 +2453,60 @@
       </c>
       <c r="K34" s="26" t="n"/>
       <c r="L34" s="25" t="inlineStr">
+        <is>
+          <t>人物特征</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>PlanetInspiredTraits</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>行星之子</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Klimter</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/klimter</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>46255</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <v>46255</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>无需前置</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>必须放第一层</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>images/klimter-planetinspiredtraits.png</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
         <is>
           <t>人物特征</t>
         </is>

</xml_diff>

<commit_message>
上新 Klimter - MoreHobbyTraits（更多爱好特征）
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2627,6 +2627,60 @@
         </is>
       </c>
       <c r="L37" t="inlineStr">
+        <is>
+          <t>人物特征</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MoreHobbyTraits</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>更多爱好特征</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Klimter</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/klimter</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>46262</v>
+      </c>
+      <c r="G38" s="16" t="n">
+        <v>46262</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>无需前置</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>必须放第一层</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>images/klimter-morehobytraits.png</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
         <is>
           <t>人物特征</t>
         </is>

</xml_diff>

<commit_message>
上新 Klimter - Immortalitytrait（永不衰老）
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2679,8 +2679,61 @@
           <t>images/klimter-morehobytraits.png</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr">
+        <is>
+          <t>人物特征</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Immortalitytrait</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>永不衰老</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Klimter</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/klimter</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>46262</v>
+      </c>
+      <c r="G39" s="16" t="n">
+        <v>46262</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>无需前置</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>必须放第一层</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>images/klimter-immortalitytrait.png</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
         <is>
           <t>人物特征</t>
         </is>

</xml_diff>

<commit_message>
新增 Klimter - PatientTrait 耐心 模组并发布
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -11,8 +11,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1133,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M40"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="10" min="1" max="1"/>
@@ -3608,7 +3609,65 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="36" customHeight="1" s="10"/>
+    <row r="41" ht="36" customHeight="1" s="10">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
+          <t>PatientTrait</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>耐心</t>
+        </is>
+      </c>
+      <c r="D41" s="8" t="inlineStr">
+        <is>
+          <t>Klimter</t>
+        </is>
+      </c>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/klimter</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t>https://www.curseforge.com/sims4/mods/patient-trait</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="n">
+        <v>46267</v>
+      </c>
+      <c r="H41" s="14" t="n">
+        <v>46267</v>
+      </c>
+      <c r="I41" s="13" t="inlineStr">
+        <is>
+          <t>无需前置</t>
+        </is>
+      </c>
+      <c r="J41" s="13" t="inlineStr">
+        <is>
+          <t>必须放第一层</t>
+        </is>
+      </c>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>images/klimter-patienttrait.png</t>
+        </is>
+      </c>
+      <c r="L41" s="8" t="n"/>
+      <c r="M41" s="13" t="inlineStr">
+        <is>
+          <t>人物特征</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="4">
     <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">

</xml_diff>

<commit_message>
新增 Klimter - Soft-HeartedTrait 心肠软弱 模组并发布
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -1133,7 +1133,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="10" min="1" max="1"/>
@@ -3662,6 +3662,65 @@
       </c>
       <c r="L41" s="8" t="n"/>
       <c r="M41" s="13" t="inlineStr">
+        <is>
+          <t>人物特征</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="36" customHeight="1" s="10">
+      <c r="A42" s="13" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>Soft-HeartedTrait</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>心肠软弱</t>
+        </is>
+      </c>
+      <c r="D42" s="8" t="inlineStr">
+        <is>
+          <t>Klimter</t>
+        </is>
+      </c>
+      <c r="E42" s="8" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/klimter</t>
+        </is>
+      </c>
+      <c r="F42" s="8" t="inlineStr">
+        <is>
+          <t>https://www.curseforge.com/sims4/mods/soft-hearted-trait</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="n">
+        <v>46269</v>
+      </c>
+      <c r="H42" s="14" t="n">
+        <v>46269</v>
+      </c>
+      <c r="I42" s="13" t="inlineStr">
+        <is>
+          <t>无需前置</t>
+        </is>
+      </c>
+      <c r="J42" s="13" t="inlineStr">
+        <is>
+          <t>必须放第一层</t>
+        </is>
+      </c>
+      <c r="K42" s="8" t="inlineStr">
+        <is>
+          <t>images/klimter-softheartedtrait.png</t>
+        </is>
+      </c>
+      <c r="L42" s="8" t="n"/>
+      <c r="M42" s="13" t="inlineStr">
         <is>
           <t>人物特征</t>
         </is>

</xml_diff>

<commit_message>
更新 Klimter MoreHobbyTraits/Immortalitytrait 百度网盘链接
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -3483,7 +3483,11 @@
           <t>images/klimter-morehobytraits.png</t>
         </is>
       </c>
-      <c r="L38" s="3" t="n"/>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>链接: https://pan.baidu.com/s/1NyT9GWICVfyLzQvtpjexMQ 提取码: hqnw</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
           <t>人物特征</t>
@@ -3542,7 +3546,11 @@
           <t>images/klimter-immortalitytrait.png</t>
         </is>
       </c>
-      <c r="L39" s="3" t="n"/>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>链接: https://pan.baidu.com/s/11FRdiNPX3V_eWde9lEdBag 提取码: zfn6</t>
+        </is>
+      </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
           <t>人物特征</t>

</xml_diff>

<commit_message>
新增 JayESims High School Tea 高中吃瓜作品
</commit_message>
<xml_diff>
--- a/作品信息.xlsx
+++ b/作品信息.xlsx
@@ -1014,7 +1014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="13" min="1" max="1"/>
@@ -3675,6 +3675,65 @@
       <c r="M43" s="23" t="inlineStr">
         <is>
           <t>人物特征</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="36" customHeight="1" s="22">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>已发布</t>
+        </is>
+      </c>
+      <c r="B44" s="24" t="inlineStr">
+        <is>
+          <t>High School Tea</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="inlineStr">
+        <is>
+          <t>高中吃瓜</t>
+        </is>
+      </c>
+      <c r="D44" s="24" t="inlineStr">
+        <is>
+          <t>JayESims</t>
+        </is>
+      </c>
+      <c r="E44" s="24" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/cw/JayESims</t>
+        </is>
+      </c>
+      <c r="F44" s="24" t="inlineStr">
+        <is>
+          <t>https://www.patreon.com/JayESims/posts/jayesims-x-jaye-139297180</t>
+        </is>
+      </c>
+      <c r="G44" s="25" t="n">
+        <v>46272</v>
+      </c>
+      <c r="H44" s="25" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I44" s="23" t="inlineStr">
+        <is>
+          <t>XML 注入器</t>
+        </is>
+      </c>
+      <c r="J44" s="23" t="inlineStr">
+        <is>
+          <t>无需放第一层</t>
+        </is>
+      </c>
+      <c r="K44" s="24" t="inlineStr">
+        <is>
+          <t>images/jayesims-high-school-tea.png</t>
+        </is>
+      </c>
+      <c r="L44" s="24" t="inlineStr"/>
+      <c r="M44" s="23" t="inlineStr">
+        <is>
+          <t>游戏玩法</t>
         </is>
       </c>
     </row>

</xml_diff>